<commit_message>
Major design overhaul has begun. Everything still W.I.P.
</commit_message>
<xml_diff>
--- a/electronics/altium_config/templates/BOM_Template.xlsx
+++ b/electronics/altium_config/templates/BOM_Template.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Projects\ROS Robot\ROS-Robot-Hardware\electronics\altium_templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Projects\ROS Robot\ROS-Robot-Hardware\electronics\altium_config\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E5C7AA9-DB3B-45C0-AF40-CC9D484978B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E0F6684-2F44-4FDB-B3B1-9CE84CC3295D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="31">
   <si>
     <t>Project File Name:</t>
   </si>
@@ -50,16 +50,43 @@
     <t>Column=Supplier Part Number 1</t>
   </si>
   <si>
-    <t>Column=Supplier Unit Price 1</t>
-  </si>
-  <si>
-    <t>Column=Manufacturer 1</t>
-  </si>
-  <si>
-    <t>Column=Manufacturer Part Number 1</t>
-  </si>
-  <si>
-    <t>Column=DesignItemId</t>
+    <t>Main Project:</t>
+  </si>
+  <si>
+    <t>Field=MainProjectName</t>
+  </si>
+  <si>
+    <t>Field=CurrentDate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Author: </t>
+  </si>
+  <si>
+    <t>Field=DrawnBy</t>
+  </si>
+  <si>
+    <t>No. Of Parts</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Date Exported: </t>
+  </si>
+  <si>
+    <t>Column=Value</t>
+  </si>
+  <si>
+    <t>Column=Voltage</t>
+  </si>
+  <si>
+    <t>Column=Color</t>
+  </si>
+  <si>
+    <t>Column=Description</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Variant: </t>
+  </si>
+  <si>
+    <t>Field=VariantName</t>
   </si>
   <si>
     <t>Part Number</t>
@@ -68,7 +95,22 @@
     <t>Description</t>
   </si>
   <si>
-    <t>Manufacture</t>
+    <t>Value</t>
+  </si>
+  <si>
+    <t>Tolerance</t>
+  </si>
+  <si>
+    <t>Voltage</t>
+  </si>
+  <si>
+    <t>Color</t>
+  </si>
+  <si>
+    <t>Quantity</t>
+  </si>
+  <si>
+    <t>Manufacturer</t>
   </si>
   <si>
     <t>Supplier</t>
@@ -77,74 +119,20 @@
     <t>Supplier Part Number</t>
   </si>
   <si>
-    <t>Supplier Unit Price</t>
-  </si>
-  <si>
-    <t>Quantity</t>
-  </si>
-  <si>
-    <t>Manufacture Part Number</t>
-  </si>
-  <si>
-    <t>Main Project:</t>
-  </si>
-  <si>
-    <t>Field=MainProjectName</t>
-  </si>
-  <si>
-    <t>Field=CurrentDate</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Author: </t>
-  </si>
-  <si>
-    <t>Field=DrawnBy</t>
-  </si>
-  <si>
-    <t>No. Of Parts</t>
-  </si>
-  <si>
-    <t>Value</t>
-  </si>
-  <si>
-    <t>Voltage</t>
-  </si>
-  <si>
-    <t>Color</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Date Exported: </t>
-  </si>
-  <si>
-    <t>Total Unit Cost</t>
-  </si>
-  <si>
-    <t>Column=Value</t>
-  </si>
-  <si>
-    <t>Column=Voltage</t>
-  </si>
-  <si>
-    <t>Column=Color</t>
-  </si>
-  <si>
-    <t>Name</t>
-  </si>
-  <si>
-    <t>Column=Name</t>
-  </si>
-  <si>
-    <t>Column=Description</t>
+    <t>Column=Part Number</t>
+  </si>
+  <si>
+    <t>Column=Tolerance</t>
+  </si>
+  <si>
+    <t>Column=Manufacturer</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-  </numFmts>
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -154,12 +142,6 @@
     </font>
     <font>
       <sz val="10"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="24"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
@@ -221,7 +203,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="23">
+  <borders count="17">
     <border>
       <left/>
       <right/>
@@ -316,19 +298,6 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left style="medium">
         <color indexed="64"/>
       </left>
@@ -342,19 +311,6 @@
     <border>
       <left/>
       <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
         <color indexed="64"/>
       </right>
       <top style="thin">
@@ -428,73 +384,13 @@
       <left style="thin">
         <color indexed="64"/>
       </left>
-      <right style="thin">
+      <right style="medium">
         <color indexed="64"/>
       </right>
       <top style="medium">
         <color indexed="64"/>
       </top>
       <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
         <color indexed="64"/>
       </bottom>
       <diagonal/>
@@ -503,9 +399,9 @@
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="53">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
@@ -513,98 +409,75 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="2" xfId="2" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="2" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="3" borderId="18" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="19" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="16" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="40% - Accent5" xfId="2" builtinId="47"/>
@@ -628,14 +501,14 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>11</xdr:col>
-      <xdr:colOff>997323</xdr:colOff>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>2196352</xdr:colOff>
       <xdr:row>2</xdr:row>
       <xdr:rowOff>54907</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>641978</xdr:colOff>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>597154</xdr:colOff>
       <xdr:row>8</xdr:row>
       <xdr:rowOff>274</xdr:rowOff>
     </xdr:to>
@@ -665,7 +538,7 @@
       </xdr:blipFill>
       <xdr:spPr bwMode="auto">
         <a:xfrm>
-          <a:off x="17100176" y="547966"/>
+          <a:off x="15419293" y="547966"/>
           <a:ext cx="1000567" cy="1099573"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -700,8 +573,8 @@
   </xdr:twoCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>1024216</xdr:colOff>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>273426</xdr:colOff>
       <xdr:row>3</xdr:row>
       <xdr:rowOff>179295</xdr:rowOff>
     </xdr:from>
@@ -719,7 +592,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="14023040" y="874060"/>
+          <a:off x="12465426" y="874060"/>
           <a:ext cx="2812677" cy="505267"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1052,285 +925,244 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M21"/>
+  <dimension ref="A1:K19"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
-    <col min="2" max="2" width="28.28515625" customWidth="1"/>
-    <col min="3" max="3" width="34.5703125" customWidth="1"/>
-    <col min="4" max="4" width="42.85546875" customWidth="1"/>
-    <col min="5" max="5" width="10.140625" customWidth="1"/>
-    <col min="6" max="7" width="10" customWidth="1"/>
-    <col min="8" max="8" width="33.85546875" customWidth="1"/>
-    <col min="9" max="9" width="28.28515625" customWidth="1"/>
-    <col min="10" max="10" width="15.28515625" customWidth="1"/>
-    <col min="11" max="11" width="29" customWidth="1"/>
-    <col min="12" max="12" width="20.28515625" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" customWidth="1"/>
+    <col min="2" max="2" width="29" customWidth="1"/>
+    <col min="3" max="3" width="63.5703125" customWidth="1"/>
+    <col min="4" max="4" width="10.5703125" customWidth="1"/>
+    <col min="5" max="5" width="9.85546875" customWidth="1"/>
+    <col min="6" max="6" width="11.7109375" customWidth="1"/>
+    <col min="7" max="7" width="9.28515625" customWidth="1"/>
+    <col min="8" max="8" width="32.7109375" customWidth="1"/>
+    <col min="9" max="9" width="15.42578125" customWidth="1"/>
+    <col min="10" max="10" width="39" customWidth="1"/>
+    <col min="11" max="11" width="12.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="20.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C1" s="1"/>
-      <c r="D1" s="22"/>
-      <c r="E1" s="22"/>
-      <c r="F1" s="22"/>
+    <row r="1" spans="1:11" ht="20.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C1" s="21"/>
+      <c r="D1" s="21"/>
+      <c r="E1" s="21"/>
+      <c r="F1" s="21"/>
       <c r="G1" s="1"/>
       <c r="H1" s="1"/>
       <c r="I1" s="1"/>
       <c r="J1" s="1"/>
-      <c r="K1" s="1"/>
-    </row>
-    <row r="2" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B2" s="13"/>
-      <c r="C2" s="10"/>
+    </row>
+    <row r="2" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="B2" s="12"/>
       <c r="G2" s="2"/>
       <c r="H2" s="2"/>
       <c r="I2" s="2"/>
       <c r="J2" s="2"/>
-      <c r="K2" s="2"/>
-      <c r="L2" s="2"/>
-      <c r="M2" s="23"/>
-    </row>
-    <row r="3" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K2" s="22"/>
+    </row>
+    <row r="3" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B3" s="5"/>
-      <c r="C3" s="3"/>
       <c r="G3" s="3"/>
       <c r="H3" s="3"/>
       <c r="I3" s="3"/>
       <c r="J3" s="3"/>
-      <c r="K3" s="3"/>
-      <c r="L3" s="3"/>
-      <c r="M3" s="24"/>
-    </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="K3" s="23"/>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" s="9"/>
-      <c r="B4" s="11" t="s">
-        <v>17</v>
-      </c>
-      <c r="C4" s="19" t="s">
-        <v>18</v>
+      <c r="B4" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4" s="18" t="s">
+        <v>6</v>
       </c>
       <c r="G4" s="3"/>
-      <c r="I4" s="3"/>
-      <c r="K4" s="3"/>
-      <c r="L4" s="3"/>
-      <c r="M4" s="24"/>
-    </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="J4" s="3"/>
+      <c r="K4" s="23"/>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" s="9"/>
-      <c r="B5" s="11" t="s">
+      <c r="B5" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="C5" s="20" t="s">
+      <c r="C5" s="19" t="s">
         <v>1</v>
       </c>
       <c r="G5" s="3"/>
-      <c r="I5" s="3"/>
-      <c r="K5" s="3"/>
-      <c r="L5" s="3"/>
-      <c r="M5" s="24"/>
-    </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="J5" s="3"/>
+      <c r="K5" s="23"/>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" s="9"/>
-      <c r="B6" s="12" t="s">
-        <v>26</v>
-      </c>
-      <c r="C6" s="21" t="s">
-        <v>19</v>
+      <c r="B6" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="C6" s="20" t="s">
+        <v>7</v>
       </c>
       <c r="G6" s="4"/>
-      <c r="I6" s="4"/>
-      <c r="K6" s="3"/>
-      <c r="L6" s="3"/>
-      <c r="M6" s="24"/>
-    </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="J6" s="3"/>
+      <c r="K6" s="23"/>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" s="9"/>
-      <c r="B7" s="12" t="s">
-        <v>20</v>
-      </c>
-      <c r="C7" s="21" t="s">
-        <v>21</v>
+      <c r="B7" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="C7" s="20" t="s">
+        <v>9</v>
       </c>
       <c r="G7" s="4"/>
       <c r="H7" s="4"/>
       <c r="I7" s="4"/>
       <c r="J7" s="4"/>
-      <c r="K7" s="4"/>
-      <c r="L7" s="4"/>
-      <c r="M7" s="9"/>
-    </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="B8" s="5"/>
-      <c r="C8" s="4"/>
+      <c r="K7" s="9"/>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A8" s="9"/>
+      <c r="B8" s="39" t="s">
+        <v>16</v>
+      </c>
+      <c r="C8" s="20" t="s">
+        <v>17</v>
+      </c>
       <c r="G8" s="4"/>
       <c r="H8" s="4"/>
       <c r="I8" s="4"/>
       <c r="J8" s="4"/>
-      <c r="K8" s="4"/>
-      <c r="L8" s="4"/>
-      <c r="M8" s="9"/>
-    </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="K8" s="9"/>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B9" s="5"/>
-      <c r="C9" s="4"/>
       <c r="G9" s="4"/>
       <c r="H9" s="4"/>
       <c r="I9" s="4"/>
       <c r="J9" s="4"/>
-      <c r="K9" s="4"/>
-      <c r="L9" s="4"/>
-      <c r="M9" s="9"/>
-    </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="K9" s="9"/>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B10" s="5"/>
-      <c r="C10" s="4"/>
       <c r="G10" s="4"/>
       <c r="H10" s="4"/>
       <c r="I10" s="4"/>
       <c r="J10" s="4"/>
-      <c r="K10" s="4"/>
-      <c r="L10" s="4"/>
-      <c r="M10" s="9"/>
-    </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="B11" s="26" t="s">
-        <v>9</v>
-      </c>
-      <c r="C11" s="27" t="s">
-        <v>31</v>
-      </c>
-      <c r="D11" s="25" t="s">
-        <v>10</v>
-      </c>
-      <c r="E11" s="25" t="s">
+      <c r="K10" s="9"/>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="B11" s="25" t="s">
+        <v>18</v>
+      </c>
+      <c r="C11" s="24" t="s">
+        <v>19</v>
+      </c>
+      <c r="D11" s="24" t="s">
+        <v>20</v>
+      </c>
+      <c r="E11" s="24" t="s">
+        <v>22</v>
+      </c>
+      <c r="F11" s="24" t="s">
+        <v>21</v>
+      </c>
+      <c r="G11" s="26" t="s">
         <v>23</v>
       </c>
-      <c r="F11" s="25" t="s">
+      <c r="H11" s="27" t="s">
+        <v>25</v>
+      </c>
+      <c r="I11" s="27" t="s">
+        <v>26</v>
+      </c>
+      <c r="J11" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="K11" s="28" t="s">
         <v>24</v>
       </c>
-      <c r="G11" s="28" t="s">
-        <v>25</v>
-      </c>
-      <c r="H11" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="I11" s="29" t="s">
-        <v>16</v>
-      </c>
-      <c r="J11" s="29" t="s">
+    </row>
+    <row r="12" spans="1:11" ht="30" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B12" s="31" t="s">
+        <v>28</v>
+      </c>
+      <c r="C12" s="32" t="s">
+        <v>15</v>
+      </c>
+      <c r="D12" s="32" t="s">
         <v>12</v>
       </c>
-      <c r="K11" s="29" t="s">
+      <c r="E12" s="32" t="s">
         <v>13</v>
       </c>
-      <c r="L11" s="29" t="s">
+      <c r="F12" s="32" t="s">
+        <v>29</v>
+      </c>
+      <c r="G12" s="33" t="s">
         <v>14</v>
       </c>
-      <c r="M11" s="30" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="12" spans="1:13" ht="30" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B12" s="35" t="s">
-        <v>8</v>
-      </c>
-      <c r="C12" s="36" t="s">
-        <v>32</v>
-      </c>
-      <c r="D12" s="37" t="s">
-        <v>33</v>
-      </c>
-      <c r="E12" s="37" t="s">
-        <v>28</v>
-      </c>
-      <c r="F12" s="37" t="s">
-        <v>29</v>
-      </c>
-      <c r="G12" s="38" t="s">
+      <c r="H12" s="33" t="s">
         <v>30</v>
       </c>
-      <c r="H12" s="38" t="s">
-        <v>6</v>
-      </c>
-      <c r="I12" s="38" t="s">
-        <v>7</v>
-      </c>
-      <c r="J12" s="38" t="s">
+      <c r="I12" s="33" t="s">
         <v>3</v>
       </c>
-      <c r="K12" s="38" t="s">
+      <c r="J12" s="33" t="s">
         <v>4</v>
       </c>
-      <c r="L12" s="38" t="s">
-        <v>5</v>
-      </c>
-      <c r="M12" s="39" t="s">
+      <c r="K12" s="34" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="B13" s="47"/>
-      <c r="C13" s="48"/>
-      <c r="D13" s="48"/>
-      <c r="E13" s="40"/>
-      <c r="F13" s="40"/>
-      <c r="G13" s="40"/>
-      <c r="H13" s="40"/>
-      <c r="I13" s="40"/>
-      <c r="J13" s="40"/>
-      <c r="K13" s="40"/>
-      <c r="L13" s="41"/>
-      <c r="M13" s="42"/>
-    </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="B14" s="49"/>
-      <c r="C14" s="50"/>
-      <c r="D14" s="50"/>
-      <c r="E14" s="43"/>
-      <c r="F14" s="43"/>
-      <c r="G14" s="43"/>
-      <c r="H14" s="43"/>
-      <c r="I14" s="43"/>
-      <c r="J14" s="43"/>
-      <c r="K14" s="43"/>
-      <c r="L14" s="43"/>
-      <c r="M14" s="44"/>
-    </row>
-    <row r="15" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="51"/>
-      <c r="C15" s="52"/>
-      <c r="D15" s="52"/>
-      <c r="E15" s="45"/>
-      <c r="F15" s="45"/>
-      <c r="G15" s="45"/>
-      <c r="H15" s="45"/>
-      <c r="I15" s="45"/>
-      <c r="J15" s="45"/>
-      <c r="K15" s="45"/>
-      <c r="L15" s="45"/>
-      <c r="M15" s="46"/>
-    </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="B16" s="16"/>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="B13" s="37"/>
+      <c r="C13" s="38"/>
+      <c r="D13" s="35"/>
+      <c r="E13" s="35"/>
+      <c r="F13" s="35"/>
+      <c r="G13" s="35"/>
+      <c r="H13" s="35"/>
+      <c r="I13" s="35"/>
+      <c r="J13" s="35"/>
+      <c r="K13" s="36"/>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="B14" s="37"/>
+      <c r="C14" s="38"/>
+      <c r="D14" s="35"/>
+      <c r="E14" s="35"/>
+      <c r="F14" s="35"/>
+      <c r="G14" s="35"/>
+      <c r="H14" s="35"/>
+      <c r="I14" s="35"/>
+      <c r="J14" s="35"/>
+      <c r="K14" s="36"/>
+    </row>
+    <row r="15" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B15" s="37"/>
+      <c r="C15" s="38"/>
+      <c r="D15" s="35"/>
+      <c r="E15" s="35"/>
+      <c r="F15" s="35"/>
+      <c r="G15" s="35"/>
+      <c r="H15" s="35"/>
+      <c r="I15" s="35"/>
+      <c r="J15" s="35"/>
+      <c r="K15" s="36"/>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="B16" s="15"/>
       <c r="C16" s="8"/>
       <c r="D16" s="8"/>
       <c r="E16" s="8"/>
       <c r="F16" s="8"/>
       <c r="G16" s="8"/>
-      <c r="H16" s="17"/>
-      <c r="I16" s="17"/>
+      <c r="H16" s="16"/>
+      <c r="I16" s="16"/>
       <c r="J16" s="17"/>
-      <c r="K16" s="18"/>
-      <c r="L16" s="33" t="s">
-        <v>27</v>
-      </c>
-      <c r="M16" s="34" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="17" spans="2:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B17" s="14"/>
+      <c r="K16" s="30" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="17" spans="2:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B17" s="13"/>
       <c r="C17" s="6"/>
       <c r="D17" s="6"/>
       <c r="E17" s="6"/>
@@ -1338,18 +1170,13 @@
       <c r="G17" s="6"/>
       <c r="H17" s="7"/>
       <c r="I17" s="7"/>
-      <c r="J17" s="7"/>
-      <c r="K17" s="15"/>
-      <c r="L17" s="31">
-        <f>SUM(L13:L15)</f>
+      <c r="J17" s="14"/>
+      <c r="K17" s="29">
+        <f>SUM(K13:K15)</f>
         <v>0</v>
       </c>
-      <c r="M17" s="32">
-        <f>SUM(M13:M15)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18" spans="2:13" x14ac:dyDescent="0.25">
+    </row>
+    <row r="18" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B18" s="4"/>
       <c r="C18" s="4"/>
       <c r="D18" s="4"/>
@@ -1358,9 +1185,8 @@
       <c r="G18" s="4"/>
       <c r="H18" s="4"/>
       <c r="I18" s="4"/>
-      <c r="J18" s="4"/>
-    </row>
-    <row r="19" spans="2:13" x14ac:dyDescent="0.25">
+    </row>
+    <row r="19" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B19" s="4"/>
       <c r="C19" s="4"/>
       <c r="D19" s="4"/>
@@ -1369,29 +1195,6 @@
       <c r="G19" s="4"/>
       <c r="H19" s="4"/>
       <c r="I19" s="4"/>
-      <c r="J19" s="4"/>
-    </row>
-    <row r="20" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B20" s="4"/>
-      <c r="C20" s="4"/>
-      <c r="D20" s="4"/>
-      <c r="E20" s="4"/>
-      <c r="F20" s="4"/>
-      <c r="G20" s="4"/>
-      <c r="H20" s="4"/>
-      <c r="I20" s="4"/>
-      <c r="J20" s="4"/>
-    </row>
-    <row r="21" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B21" s="4"/>
-      <c r="C21" s="4"/>
-      <c r="D21" s="4"/>
-      <c r="E21" s="4"/>
-      <c r="F21" s="4"/>
-      <c r="G21" s="4"/>
-      <c r="H21" s="4"/>
-      <c r="I21" s="4"/>
-      <c r="J21" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>